<commit_message>
excel write data fixed
</commit_message>
<xml_diff>
--- a/dynamics/src/dynamics/dynamics_calc.xlsx
+++ b/dynamics/src/dynamics/dynamics_calc.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,6 +468,66 @@
         <v>0</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>0</v>
+      </c>
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E3" t="n">
+        <v>4</v>
+      </c>
+      <c r="F3" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B4" t="n">
+        <v>7</v>
+      </c>
+      <c r="C4" t="n">
+        <v>8</v>
+      </c>
+      <c r="D4" t="n">
+        <v>9</v>
+      </c>
+      <c r="E4" t="n">
+        <v>10</v>
+      </c>
+      <c r="F4" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>12</v>
+      </c>
+      <c r="B5" t="n">
+        <v>13</v>
+      </c>
+      <c r="C5" t="n">
+        <v>14</v>
+      </c>
+      <c r="D5" t="n">
+        <v>15</v>
+      </c>
+      <c r="E5" t="n">
+        <v>16</v>
+      </c>
+      <c r="F5" t="n">
+        <v>17</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
 </worksheet>

</xml_diff>

<commit_message>
fixed xlsx & picture save
</commit_message>
<xml_diff>
--- a/dynamics/src/dynamics/dynamics_calc.xlsx
+++ b/dynamics/src/dynamics/dynamics_calc.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -466,66 +466,6 @@
       </c>
       <c r="F2" t="n">
         <v>0</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>0</v>
-      </c>
-      <c r="B3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D3" t="n">
-        <v>3</v>
-      </c>
-      <c r="E3" t="n">
-        <v>4</v>
-      </c>
-      <c r="F3" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>6</v>
-      </c>
-      <c r="B4" t="n">
-        <v>7</v>
-      </c>
-      <c r="C4" t="n">
-        <v>8</v>
-      </c>
-      <c r="D4" t="n">
-        <v>9</v>
-      </c>
-      <c r="E4" t="n">
-        <v>10</v>
-      </c>
-      <c r="F4" t="n">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>12</v>
-      </c>
-      <c r="B5" t="n">
-        <v>13</v>
-      </c>
-      <c r="C5" t="n">
-        <v>14</v>
-      </c>
-      <c r="D5" t="n">
-        <v>15</v>
-      </c>
-      <c r="E5" t="n">
-        <v>16</v>
-      </c>
-      <c r="F5" t="n">
-        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>